<commit_message>
Correct BHRaSYC to put all existing capacity in the 2020 column
</commit_message>
<xml_diff>
--- a/InputData/elec/BHRaSYC/BAU Heat Rates and Start Year Capacities.xlsx
+++ b/InputData/elec/BHRaSYC/BAU Heat Rates and Start Year Capacities.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\MeganMahajan\Documents\eps-india\InputData\elec\BHRaSYC\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1354C40F-89A6-4BB2-A87D-F9FC6C10F57E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0376A1D3-EAB1-4A66-9E21-EE1360CCD0B6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="17520" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="17520" activeTab="4" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="About" sheetId="1" r:id="rId1"/>
@@ -24944,25 +24944,21 @@
       <c r="DW2">
         <v>0</v>
       </c>
-      <c r="DX2" s="5">
-        <f>'Start Year Capacities - 2026-21'!F8</f>
-        <v>192971.5</v>
-      </c>
-      <c r="DY2" s="5">
-        <f>'Start Year Capacities - 2026-21'!E8</f>
-        <v>191092.5</v>
-      </c>
-      <c r="DZ2" s="5">
-        <f>'Start Year Capacities - 2026-21'!D8</f>
-        <v>198494.5</v>
+      <c r="DX2">
+        <v>0</v>
+      </c>
+      <c r="DY2">
+        <v>0</v>
+      </c>
+      <c r="DZ2">
+        <v>0</v>
       </c>
       <c r="EA2">
         <f>'Start Year Capacities - 2026-21'!C8</f>
         <v>199864.5</v>
       </c>
       <c r="EB2">
-        <f>'Start Year Capacities - 2026-21'!J8</f>
-        <v>203189.5</v>
+        <v>0</v>
       </c>
       <c r="EC2">
         <v>0</v>
@@ -25584,25 +25580,21 @@
       <c r="DW3">
         <v>0</v>
       </c>
-      <c r="DX3" s="5">
-        <f>'Start Year Capacities - 2026-21'!E10-'BHRaSYC-StartYearCapacities'!DX4</f>
-        <v>24587.22</v>
+      <c r="DX3">
+        <v>0</v>
       </c>
       <c r="DY3">
-        <f>$DX$3/($DX$3+$DX$4)*'Start Year Capacities - 2026-21'!E10</f>
-        <v>24587.22</v>
+        <v>0</v>
       </c>
       <c r="DZ3">
-        <f>$DX$3/($DX$3+$DX$4)*'Start Year Capacities - 2026-21'!D10</f>
-        <v>24587.22</v>
-      </c>
-      <c r="EA3">
-        <f>$DX$3/($DX$3+$DX$4)*'Start Year Capacities - 2026-21'!C10</f>
-        <v>24606.239260118007</v>
+        <v>0</v>
+      </c>
+      <c r="EA3" s="5">
+        <f>'Start Year Capacities - 2026-21'!C10-EA4</f>
+        <v>24606.51</v>
       </c>
       <c r="EB3">
-        <f>$DX$3/($DX$3+$DX$4)*'Start Year Capacities - 2026-21'!J10</f>
-        <v>24550.039269100565</v>
+        <v>0</v>
       </c>
       <c r="EC3">
         <v>0</v>
@@ -26225,23 +26217,19 @@
         <v>0</v>
       </c>
       <c r="DX4">
+        <v>0</v>
+      </c>
+      <c r="DY4">
+        <v>0</v>
+      </c>
+      <c r="DZ4">
+        <v>0</v>
+      </c>
+      <c r="EA4">
         <v>350</v>
       </c>
-      <c r="DY4">
-        <f>$DX$4/($DX$3+$DX$4)*$DY$3</f>
-        <v>345.08766414219389</v>
-      </c>
-      <c r="DZ4">
-        <f t="shared" ref="DZ4:EB4" si="0">$DX$4/($DX$3+$DX$4)*$DY$3</f>
-        <v>345.08766414219389</v>
-      </c>
-      <c r="EA4">
-        <f t="shared" si="0"/>
-        <v>345.08766414219389</v>
-      </c>
       <c r="EB4">
-        <f t="shared" si="0"/>
-        <v>345.08766414219389</v>
+        <v>0</v>
       </c>
       <c r="EC4">
         <v>0</v>
@@ -26863,25 +26851,21 @@
       <c r="DW5">
         <v>0</v>
       </c>
-      <c r="DX5" s="5">
-        <f>'Start Year Capacities - 2026-21'!F12</f>
-        <v>6780</v>
-      </c>
-      <c r="DY5" s="5">
-        <f>'Start Year Capacities - 2026-21'!E12</f>
-        <v>6780</v>
-      </c>
-      <c r="DZ5" s="5">
-        <f>'Start Year Capacities - 2026-21'!D12</f>
-        <v>6780</v>
+      <c r="DX5">
+        <v>0</v>
+      </c>
+      <c r="DY5">
+        <v>0</v>
+      </c>
+      <c r="DZ5">
+        <v>0</v>
       </c>
       <c r="EA5">
         <f>'Start Year Capacities - 2026-21'!C12</f>
         <v>6780</v>
       </c>
       <c r="EB5">
-        <f>'Start Year Capacities - 2026-21'!J12</f>
-        <v>6780</v>
+        <v>0</v>
       </c>
       <c r="EC5">
         <v>0</v>
@@ -27503,25 +27487,21 @@
       <c r="DW6">
         <v>0</v>
       </c>
-      <c r="DX6" s="5">
-        <f>'Start Year Capacities - 2026-21'!F13</f>
-        <v>44963.42</v>
-      </c>
-      <c r="DY6" s="5">
-        <f>'Start Year Capacities - 2026-21'!E13</f>
-        <v>45399.22</v>
-      </c>
-      <c r="DZ6" s="5">
-        <f>'Start Year Capacities - 2026-21'!D13</f>
-        <v>45399.22</v>
+      <c r="DX6">
+        <v>0</v>
+      </c>
+      <c r="DY6">
+        <v>0</v>
+      </c>
+      <c r="DZ6">
+        <v>0</v>
       </c>
       <c r="EA6" s="8">
         <f>'Start Year Capacities - 2026-21'!C13</f>
         <v>45798.22</v>
       </c>
       <c r="EB6">
-        <f>'Start Year Capacities - 2026-21'!J13</f>
-        <v>46512.22</v>
+        <v>0</v>
       </c>
       <c r="EC6">
         <v>0</v>
@@ -28143,25 +28123,21 @@
       <c r="DW7">
         <v>0</v>
       </c>
-      <c r="DX7" s="5">
-        <f>'Start Year Capacities - 2026-21'!F15</f>
-        <v>32848.46</v>
-      </c>
-      <c r="DY7" s="5">
-        <f>'Start Year Capacities - 2026-21'!E15</f>
-        <v>35138.15</v>
-      </c>
-      <c r="DZ7" s="5">
-        <f>'Start Year Capacities - 2026-21'!D15</f>
-        <v>37505.18</v>
+      <c r="DX7">
+        <v>0</v>
+      </c>
+      <c r="DY7">
+        <v>0</v>
+      </c>
+      <c r="DZ7">
+        <v>0</v>
       </c>
       <c r="EA7">
         <f>'Start Year Capacities - 2026-21'!C15</f>
         <v>38624.15</v>
       </c>
       <c r="EB7">
-        <f>'Start Year Capacities - 2026-21'!J15</f>
-        <v>40082.699999999997</v>
+        <v>0</v>
       </c>
       <c r="EC7">
         <v>0</v>
@@ -28783,25 +28759,21 @@
       <c r="DW8">
         <v>0</v>
       </c>
-      <c r="DX8" s="5">
-        <f>'Start Year Capacities - 2026-21'!F14</f>
-        <v>17052.41</v>
-      </c>
-      <c r="DY8" s="5">
-        <f>'Start Year Capacities - 2026-21'!E14</f>
-        <v>25212.26</v>
-      </c>
-      <c r="DZ8" s="5">
-        <f>'Start Year Capacities - 2026-21'!D14</f>
-        <v>33730.559999999998</v>
+      <c r="DX8">
+        <v>0</v>
+      </c>
+      <c r="DY8">
+        <v>0</v>
+      </c>
+      <c r="DZ8">
+        <v>0</v>
       </c>
       <c r="EA8">
         <f>'Start Year Capacities - 2026-21'!C14</f>
         <v>37464.639999999999</v>
       </c>
       <c r="EB8">
-        <f>'Start Year Capacities - 2026-21'!J14</f>
-        <v>49346.71</v>
+        <v>0</v>
       </c>
       <c r="EC8">
         <v>0</v>
@@ -30058,25 +30030,21 @@
       <c r="DW10">
         <v>0</v>
       </c>
-      <c r="DX10" s="5">
-        <f>'Start Year Capacities - 2026-21'!F16</f>
-        <v>8413.7999999999993</v>
-      </c>
-      <c r="DY10" s="5">
-        <f>'Start Year Capacities - 2026-21'!E16</f>
-        <v>9075.5</v>
-      </c>
-      <c r="DZ10" s="5">
-        <f>'Start Year Capacities - 2026-21'!D16</f>
-        <v>9861.31</v>
+      <c r="DX10">
+        <v>0</v>
+      </c>
+      <c r="DY10">
+        <v>0</v>
+      </c>
+      <c r="DZ10">
+        <v>0</v>
       </c>
       <c r="EA10">
         <f>'Start Year Capacities - 2026-21'!C16</f>
         <v>10145.92</v>
       </c>
       <c r="EB10">
-        <f>'Start Year Capacities - 2026-21'!J16</f>
-        <v>10175.61</v>
+        <v>0</v>
       </c>
       <c r="EC10">
         <v>0</v>
@@ -30698,24 +30666,21 @@
       <c r="DW11">
         <v>0</v>
       </c>
-      <c r="DX11" s="5">
-        <f>'Start Year Capacities - 2026-21'!F17</f>
-        <v>4418.1499999999996</v>
-      </c>
-      <c r="DY11" s="5">
-        <f>'Start Year Capacities - 2026-21'!E17</f>
-        <v>4517.45</v>
-      </c>
-      <c r="DZ11" s="5">
-        <f>'Start Year Capacities - 2026-21'!D17</f>
-        <v>4671.5600000000004</v>
+      <c r="DX11">
+        <v>0</v>
+      </c>
+      <c r="DY11">
+        <v>0</v>
+      </c>
+      <c r="DZ11">
+        <v>0</v>
       </c>
       <c r="EA11" s="13">
         <f>'Start Year Capacities - 2026-21'!C17</f>
         <v>4750.46</v>
       </c>
       <c r="EB11">
-        <v>4744.3474133413583</v>
+        <v>0</v>
       </c>
       <c r="EC11">
         <v>0</v>
@@ -31337,25 +31302,21 @@
       <c r="DW12">
         <v>0</v>
       </c>
-      <c r="DX12" s="5">
-        <f>'Start Year Capacities - 2026-21'!F11</f>
-        <v>837.63</v>
-      </c>
-      <c r="DY12" s="5">
-        <f>'Start Year Capacities - 2026-21'!E11</f>
-        <v>637.63</v>
-      </c>
-      <c r="DZ12" s="5">
-        <f>'Start Year Capacities - 2026-21'!D11</f>
-        <v>509.71</v>
+      <c r="DX12">
+        <v>0</v>
+      </c>
+      <c r="DY12">
+        <v>0</v>
+      </c>
+      <c r="DZ12">
+        <v>0</v>
       </c>
       <c r="EA12">
         <f>'Start Year Capacities - 2026-21'!C11</f>
         <v>509.71</v>
       </c>
       <c r="EB12">
-        <f>'Start Year Capacities - 2026-21'!J11</f>
-        <v>509.71</v>
+        <v>0</v>
       </c>
       <c r="EC12">
         <v>0</v>
@@ -32612,25 +32573,21 @@
       <c r="DW14">
         <v>0</v>
       </c>
-      <c r="DX14" s="5">
-        <f>'Start Year Capacities - 2026-21'!F9</f>
-        <v>0</v>
-      </c>
-      <c r="DY14" s="5">
-        <f>'Start Year Capacities - 2026-21'!E9</f>
-        <v>6360</v>
-      </c>
-      <c r="DZ14" s="5">
-        <f>'Start Year Capacities - 2026-21'!D9</f>
-        <v>6760</v>
+      <c r="DX14">
+        <v>0</v>
+      </c>
+      <c r="DY14">
+        <v>0</v>
+      </c>
+      <c r="DZ14">
+        <v>0</v>
       </c>
       <c r="EA14">
         <f>'Start Year Capacities - 2026-21'!C9</f>
         <v>6260</v>
       </c>
       <c r="EB14">
-        <f>'Start Year Capacities - 2026-21'!J9</f>
-        <v>6620</v>
+        <v>0</v>
       </c>
       <c r="EC14">
         <v>0</v>
@@ -35157,24 +35114,21 @@
       <c r="DW18">
         <v>0</v>
       </c>
-      <c r="DX18" s="5">
-        <f>'Start Year Capacities - 2026-21'!F18</f>
-        <v>114.08</v>
-      </c>
-      <c r="DY18" s="5">
-        <f>'Start Year Capacities - 2026-21'!E18</f>
-        <v>138.30000000000001</v>
-      </c>
-      <c r="DZ18" s="5">
-        <f>'Start Year Capacities - 2026-21'!F18</f>
-        <v>114.08</v>
+      <c r="DX18">
+        <v>0</v>
+      </c>
+      <c r="DY18">
+        <v>0</v>
+      </c>
+      <c r="DZ18">
+        <v>0</v>
       </c>
       <c r="EA18" s="5">
         <f>'Start Year Capacities - 2026-21'!G18</f>
         <v>90.58</v>
       </c>
       <c r="EB18">
-        <v>434.11</v>
+        <v>0</v>
       </c>
       <c r="EC18">
         <v>0</v>
@@ -39866,9 +39820,12 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement/>
-</p:properties>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
 </file>
 
 <file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
@@ -40016,19 +39973,15 @@
 </file>
 
 <file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement/>
+</p:properties>
 </file>
 
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{0121FE85-B93F-413B-B322-A65D31F49F07}">
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{F90E0FF2-CB08-4E88-939D-374B44211EF1}">
   <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
 </file>
@@ -40052,9 +40005,10 @@
 </file>
 
 <file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{F90E0FF2-CB08-4E88-939D-374B44211EF1}">
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{0121FE85-B93F-413B-B322-A65D31F49F07}">
   <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
 </file>
</xml_diff>